<commit_message>
ajustes de tamaños de ventanas
</commit_message>
<xml_diff>
--- a/lista_eventos_cgi600.xlsx
+++ b/lista_eventos_cgi600.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bizland365-my.sharepoint.com/personal/simon_vargas_bizland_tech/Documents/val_log_reader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FBFD2661-B36C-44C7-9382-90EB642727E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="152" documentId="8_{FBFD2661-B36C-44C7-9382-90EB642727E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B152D6DF-5071-434E-B76D-A087B1167AF9}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-48" windowWidth="23256" windowHeight="12456" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3CD72D0F-0109-4709-BAE3-D4DAF02C6335}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="105">
   <si>
     <t>ID</t>
   </si>
@@ -162,6 +162,201 @@
   </si>
   <si>
     <t>Identificador de tabla y versión</t>
+  </si>
+  <si>
+    <t>Current speed: * km/h</t>
+  </si>
+  <si>
+    <t>velocidad movil</t>
+  </si>
+  <si>
+    <t>PING 8.8.8.8: SUCCESS</t>
+  </si>
+  <si>
+    <t>comunicación éxito</t>
+  </si>
+  <si>
+    <t>Update ConnectionObserver: VALIDATOR_ON</t>
+  </si>
+  <si>
+    <t>comunicación con validador</t>
+  </si>
+  <si>
+    <t>PING 8.8.8.8: FAIL</t>
+  </si>
+  <si>
+    <t>comunicacion falla</t>
+  </si>
+  <si>
+    <t>Consultando versiones…</t>
+  </si>
+  <si>
+    <t>Tabla:AL id:11 currVersion:43150</t>
+  </si>
+  <si>
+    <t>Tabla:RL id:9 currVersion:20533</t>
+  </si>
+  <si>
+    <t>Tabla:WK id:7 currVersion:147</t>
+  </si>
+  <si>
+    <t>Tabla:CP id:8 currVersion:14</t>
+  </si>
+  <si>
+    <t>Tabla:OP id:10 currVersion:1</t>
+  </si>
+  <si>
+    <t>Tabla:LI id:18 currVersion:96</t>
+  </si>
+  <si>
+    <t>Tabla:SG id:20 currVersion:80</t>
+  </si>
+  <si>
+    <t>Tabla:GP id:1 currVersion:170</t>
+  </si>
+  <si>
+    <t>Tabla:RS id:16 currVersion:72</t>
+  </si>
+  <si>
+    <t>Tabla:LR id:23 currVersion:32</t>
+  </si>
+  <si>
+    <t>Tabla:CD id:15 currVersion:85</t>
+  </si>
+  <si>
+    <t>Tabla:CO id:3 currVersion:102</t>
+  </si>
+  <si>
+    <t>Current speed: 0 km/h</t>
+  </si>
+  <si>
+    <t>detencion/parada</t>
+  </si>
+  <si>
+    <t>TARIFA SELECCIONADA=</t>
+  </si>
+  <si>
+    <t>buffer: {"key":2,"screen":3}</t>
+  </si>
+  <si>
+    <t>[UpdateHandler][T]State: RECEIVE_DATA</t>
+  </si>
+  <si>
+    <t>inicio pago?</t>
+  </si>
+  <si>
+    <t>[ConsoleInterpreter][I]Seteo etapa actual: 1</t>
+  </si>
+  <si>
+    <t>etapa 1</t>
+  </si>
+  <si>
+    <t>rateSelected: 2</t>
+  </si>
+  <si>
+    <t>rango de precio</t>
+  </si>
+  <si>
+    <t>[26/04/23-06:59:13.526][RateFile][I]En o después de 2025/12/19: retorno futureAmount 134825</t>
+  </si>
+  <si>
+    <t>tarifa seteada desde consola 2, tarifa seteada 134825</t>
+  </si>
+  <si>
+    <t>SetFare:134825</t>
+  </si>
+  <si>
+    <t>State change request: 3</t>
+  </si>
+  <si>
+    <t>[State][T]Ready to doValidate!</t>
+  </si>
+  <si>
+    <t>TARIFA SELECCIONADA=2</t>
+  </si>
+  <si>
+    <t>[thread 3224]wake up !!</t>
+  </si>
+  <si>
+    <t>Estado de la consola: 18. Estado del validador: 3</t>
+  </si>
+  <si>
+    <t>presente tarjeta en validador</t>
+  </si>
+  <si>
+    <t>[thread 4004]EVENTO DE COBRO --&gt; fareId:30 --&gt; monto:134825</t>
+  </si>
+  <si>
+    <t>cobro pasaje</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[thread 4004]Nueva transacción. Perfil: 4 </t>
+  </si>
+  <si>
+    <t>cobro por mifare exitoso</t>
+  </si>
+  <si>
+    <t>Seteando período de logueo de dia con servicio activo</t>
+  </si>
+  <si>
+    <t>preparado para realizar cobro</t>
+  </si>
+  <si>
+    <t>No hay update pendiente</t>
+  </si>
+  <si>
+    <t>fin de descarga de Parametria nueva. No hay novedad.</t>
+  </si>
+  <si>
+    <t>Descarga parametria EXITO</t>
+  </si>
+  <si>
+    <t>descarga de Parametria exitosa</t>
+  </si>
+  <si>
+    <t>&lt;-- taskDescargaParametria()</t>
+  </si>
+  <si>
+    <t>--&gt; taskDescargaParametria()</t>
+  </si>
+  <si>
+    <t>[ConnectionObserver][T][thread 3871]Update ConnectionObserver: VALIDATOR_ON</t>
+  </si>
+  <si>
+    <t>inicio rutina de descarga de nueva parametria desde servidor Trackme (c/60 min)</t>
+  </si>
+  <si>
+    <t>[timestamp][FeedbackSubject][T][thread 3871]PING 8.8.8.8: SUCCESS SUCCESS
+[timestamp][FeedbackSubject][T][thread 3871]netstat -an | grep '200.51.194.194:19204'  - ret size 2
+[timestamp][FeedbackSubject][T][thread 3871]connectionState: CONEXION_OK  lastconnectionState: CONEXION_OK</t>
+  </si>
+  <si>
+    <t>monitoreo de conectividad y salud de red del validador. Verifica que el "túnel" de comunicación hacia el exterior esté abierto y funcionando.                                                                                                               (1ro)Ping de Google (8.8.8.8): El sistema lanza un "ping" al DNS de Google para verificar si tiene salida a Internet. El resultado es SUCCESS, lo que confirma que el módem (posiblemente el Quectel que mencionamos antes) tiene señal y acceso a la red pública.
+(2do)Verificación de Socket Específico: Ejecuta un comando de Linux (netstat) para ver si hay una conexión activa hacia la IP 200.51.194.194 en el puerto 19204.
+Esta IP pertenece probablemente al servidor central de RedBus o al concentrador de transacciones.
+El ret size 2 indica que encontró líneas de conexión (probablemente una en estado ESTABLISHED).
+(3ro)Actualización de Estado: Al confirmar que ambos puntos responden, el sistema setea internamente el connectionState como CONEXION_OK</t>
+  </si>
+  <si>
+    <t>[FeedbackSubject][T][thread 3871]valconnectionState CHANGED!: VALIDATOR_OFF</t>
+  </si>
+  <si>
+    <t>[ConnectionObserver][T][thread 3871]Update ConnectionObserver: VALIDATOR_OFF</t>
+  </si>
+  <si>
+    <t>[FeedbackSubject][T][thread 3871]valconnectionState CHANGED!: VALIDATOR_ON</t>
+  </si>
+  <si>
+    <t>nuevo estado validador: APAGADO</t>
+  </si>
+  <si>
+    <t>nuevo estado validador: ENCENDIDO</t>
+  </si>
+  <si>
+    <t>estado: APAGADO</t>
+  </si>
+  <si>
+    <t>estado: ENCENDIDO</t>
   </si>
 </sst>
 </file>
@@ -185,7 +380,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -325,23 +520,43 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -677,454 +892,695 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B1D1B55-AF86-45B6-9E5B-2D3BFD69756D}">
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="60.36328125" customWidth="1"/>
-    <col min="3" max="3" width="78.90625" customWidth="1"/>
+    <col min="1" max="1" width="10.90625" style="5"/>
+    <col min="2" max="2" width="102" style="5" customWidth="1"/>
+    <col min="3" max="3" width="78.90625" style="5" customWidth="1"/>
+    <col min="4" max="16384" width="10.90625" style="5"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2" s="5">
+      <c r="A2" s="6">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="8" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="7">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="3"/>
+      <c r="B3" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="7">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="3"/>
+      <c r="B4" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>45</v>
+      </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="7">
+      <c r="A5" s="9"/>
+      <c r="B5" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="8"/>
-      <c r="C5" s="3"/>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6" s="7">
+      <c r="B6" s="10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A7" s="9">
         <v>5</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="3"/>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7" s="7">
+      <c r="B7" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="11"/>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A8" s="9">
         <v>6</v>
       </c>
-      <c r="B7" s="8"/>
-      <c r="C7" s="3"/>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8" s="7">
+      <c r="B8" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C8" s="11"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A9" s="9">
         <v>7</v>
       </c>
-      <c r="B8" s="8"/>
-      <c r="C8" s="3"/>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9" s="7">
+      <c r="B9" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="11"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A10" s="9">
         <v>8</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="3"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10" s="7">
+      <c r="B10" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" s="11"/>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A11" s="9">
         <v>9</v>
       </c>
-      <c r="B10" s="8"/>
-      <c r="C10" s="3"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11" s="7">
+      <c r="B11" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" s="11"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A12" s="9">
         <v>10</v>
       </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12" s="7">
+      <c r="B12" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="11"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A13" s="9"/>
+      <c r="B13" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="11"/>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A14" s="9"/>
+      <c r="B14" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C14" s="11"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A15" s="9"/>
+      <c r="B15" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="11"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A16" s="9"/>
+      <c r="B16" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="11"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A17" s="9"/>
+      <c r="B17" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="C17" s="11"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A18" s="9"/>
+      <c r="B18" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C18" s="11"/>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A19" s="9"/>
+      <c r="B19" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C19" s="11"/>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A20" s="9"/>
+      <c r="B20" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C20" s="11"/>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A21" s="9">
+        <v>12</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A22" s="9">
+        <v>13</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="11"/>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A23" s="9">
+        <v>14</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="11"/>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A24" s="9">
+        <v>15</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="11"/>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A25" s="9">
+        <v>16</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C25" s="11" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A27" s="9">
+        <v>18</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="C27" s="11"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A28" s="9">
+        <v>19</v>
+      </c>
+      <c r="B28" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="C28" s="11"/>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A29" s="9">
+        <v>20</v>
+      </c>
+      <c r="B29" s="10" t="s">
+        <v>67</v>
+      </c>
+      <c r="C29" s="11" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A30" s="9"/>
+      <c r="B30" s="10" t="s">
+        <v>69</v>
+      </c>
+      <c r="C30" s="11" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A31" s="9"/>
+      <c r="B31" s="10" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A32" s="9"/>
+      <c r="B32" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="C32" s="11"/>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A33" s="9"/>
+      <c r="B33" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="C33" s="11"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A34" s="9"/>
+      <c r="B34" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="11"/>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A35" s="9"/>
+      <c r="B35" s="10" t="s">
+        <v>76</v>
+      </c>
+      <c r="C35" s="11"/>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A36" s="9"/>
+      <c r="B36" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" s="11"/>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A37" s="9">
+        <v>21</v>
+      </c>
+      <c r="B37" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="8"/>
-      <c r="C12" s="3"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A13" s="7">
+      <c r="C37" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A14" s="7">
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A38" s="9">
+        <v>22</v>
+      </c>
+      <c r="B38" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>4</v>
-      </c>
-      <c r="C14" s="3"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A15" s="7">
+      <c r="C38" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="8" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="3"/>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A16" s="7">
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A39" s="9">
+        <v>17</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="C39" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A40" s="9">
+        <v>24</v>
+      </c>
+      <c r="B40" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B16" s="8" t="s">
-        <v>8</v>
-      </c>
-      <c r="C16" s="3"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="7">
+      <c r="C40" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="3"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A18" s="7">
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A41" s="9">
+        <v>25</v>
+      </c>
+      <c r="B41" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A19" s="7">
+      <c r="C41" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="8"/>
-      <c r="C19" s="3"/>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A20" s="7">
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A42" s="9">
+        <v>26</v>
+      </c>
+      <c r="B42" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B20" s="8"/>
-      <c r="C20" s="3"/>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A21" s="7">
+      <c r="C42" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B21" s="8"/>
-      <c r="C21" s="3"/>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A22" s="7">
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A43" s="9">
+        <v>27</v>
+      </c>
+      <c r="B43" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C43" s="11"/>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A44" s="9"/>
+      <c r="B44" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="11" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A45" s="9">
+        <v>28</v>
+      </c>
+      <c r="B45" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B22" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A23" s="7">
+      <c r="C45" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A24" s="7">
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A46" s="9">
+        <v>29</v>
+      </c>
+      <c r="B46" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B24" s="8"/>
-      <c r="C24" s="3"/>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A25" s="7">
+      <c r="C46" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A26" s="7">
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A47" s="9">
+        <v>30</v>
+      </c>
+      <c r="B47" s="10"/>
+      <c r="C47" s="11"/>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A48" s="9">
+        <v>31</v>
+      </c>
+      <c r="B48" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A27" s="7">
+      <c r="C48" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A28" s="7">
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A49" s="9">
+        <v>32</v>
+      </c>
+      <c r="B49" s="10"/>
+      <c r="C49" s="11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A50" s="9">
+        <v>33</v>
+      </c>
+      <c r="B50" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="8"/>
-      <c r="C28" s="3"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A29" s="7">
+      <c r="C50" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A30" s="7">
-        <v>29</v>
-      </c>
-      <c r="B30" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A31" s="7">
-        <v>30</v>
-      </c>
-      <c r="B31" s="8"/>
-      <c r="C31" s="3"/>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A32" s="7">
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A51" s="9">
+        <v>34</v>
+      </c>
+      <c r="B51" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="C51" s="11"/>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A52" s="9">
+        <v>35</v>
+      </c>
+      <c r="B52" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A53" s="9">
+        <v>36</v>
+      </c>
+      <c r="B53" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="C53" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A54" s="9">
+        <v>37</v>
+      </c>
+      <c r="B54" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A55" s="9">
+        <v>38</v>
+      </c>
+      <c r="B55" s="10"/>
+      <c r="C55" s="11"/>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A56" s="9">
+        <v>39</v>
+      </c>
+      <c r="B56" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B32" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A33" s="7">
+      <c r="C56" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A57" s="9">
+        <v>40</v>
+      </c>
+      <c r="B57" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="B33" s="8"/>
-      <c r="C33" s="3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A34" s="7">
+      <c r="C57" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A58" s="9">
+        <v>41</v>
+      </c>
+      <c r="B58" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>27</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A35" s="7">
+      <c r="C58" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A59" s="9">
+        <v>42</v>
+      </c>
+      <c r="B59" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="B35" s="8"/>
-      <c r="C35" s="3"/>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A36" s="7">
+      <c r="C59" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A60" s="9">
+        <v>43</v>
+      </c>
+      <c r="B60" s="10" t="s">
         <v>35</v>
       </c>
-      <c r="B36" s="8"/>
-      <c r="C36" s="3"/>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A37" s="7">
+      <c r="C60" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A61" s="9">
+        <v>44</v>
+      </c>
+      <c r="B61" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="B37" s="8"/>
-      <c r="C37" s="3"/>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A38" s="7">
+      <c r="C61" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A62" s="9">
+        <v>45</v>
+      </c>
+      <c r="B62" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="B38" s="8"/>
-      <c r="C38" s="3"/>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A39" s="7">
+      <c r="C62" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A63" s="9">
+        <v>46</v>
+      </c>
+      <c r="B63" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B39" s="8"/>
-      <c r="C39" s="3"/>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A40" s="7">
+      <c r="C63" s="13" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A64" s="9">
+        <v>47</v>
+      </c>
+      <c r="B64" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="B40" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C40" s="9" t="s">
+      <c r="C64" s="13" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A41" s="7">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A65" s="9">
+        <v>48</v>
+      </c>
+      <c r="B65" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="B41" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C41" s="9" t="s">
+      <c r="C65" s="13" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A42" s="7">
-        <v>41</v>
-      </c>
-      <c r="B42" s="8" t="s">
-        <v>33</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A43" s="7">
-        <v>42</v>
-      </c>
-      <c r="B43" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C43" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A44" s="7">
-        <v>43</v>
-      </c>
-      <c r="B44" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C44" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A45" s="7">
-        <v>44</v>
-      </c>
-      <c r="B45" s="8" t="s">
-        <v>36</v>
-      </c>
-      <c r="C45" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A46" s="7">
-        <v>45</v>
-      </c>
-      <c r="B46" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A47" s="7">
-        <v>46</v>
-      </c>
-      <c r="B47" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="C47" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A48" s="7">
-        <v>47</v>
-      </c>
-      <c r="B48" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C48" s="9" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A49" s="7">
-        <v>48</v>
-      </c>
-      <c r="B49" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="C49" s="9" t="s">
-        <v>41</v>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B66" s="14" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" ht="188.5" x14ac:dyDescent="0.35">
+      <c r="B67" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="C67" s="15" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B68" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="C68" s="5" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B69" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B70" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B71" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B72" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C72" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B73" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C73" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B74" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C74" s="5" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="B75" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="C75" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>